<commit_message>
Reports: add previous and current descriptions
</commit_message>
<xml_diff>
--- a/data/Reports.xlsx
+++ b/data/Reports.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5FF44F-2907-4B90-A011-88D3CD122BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096DEF2F-A5BF-4D57-B1D6-78AEA94E2ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="296">
   <si>
     <t>Year</t>
   </si>
@@ -845,6 +845,72 @@
   </si>
   <si>
     <t>Start Date</t>
+  </si>
+  <si>
+    <t>Previously: scattered, dry, and unhealthy random trees with invasive and dried weeds</t>
+  </si>
+  <si>
+    <t>After clearing the site and preparing the soil, 40 Delonix regia trees were planted. Planting beds were defined and landscaped with Sphagneticola trilobata as ground cover, bordered with Alternanthera. Seasonal Catharanthus roseus flowers and decorative cacti were also added</t>
+  </si>
+  <si>
+    <t>Site redevelopment and rehabilitation in line with modern landscaping standards to improve operational efficiency.</t>
+  </si>
+  <si>
+    <t>Landscaping was implemented across three levels:
+Upper level: a roundabout hedge of dwarf Bougainvillea.
+Middle level: a mixed-color Bougainvillea hedge.
+Lower level: ground cover using Alternanthera, enhanced with selected ornamental plants and cacti in the lower beds.</t>
+  </si>
+  <si>
+    <t>Site development and beautification in line with modern landscaping standards</t>
+  </si>
+  <si>
+    <t>The area was redesigned into defined planting beds and seating spaces. Landscaping included cacti, Ficus microcarpa (Ficus Panda), Cycas revoluta, dwarf Dracaena trifasciata varieties, with ground cover using Alternanthera and Sphagneticola trilobata</t>
+  </si>
+  <si>
+    <t>Trees were pruned and reshaped to eliminate overlap and improve safety. The area was cleared of debris, the landscaped area was expanded in an organized manner, and the overall streetscape aesthetics were enhanced.</t>
+  </si>
+  <si>
+    <t>All debris was removed, the soil was prepared and fertilized, and a new irrigation system was installed within the roundabout. A Albizia lebbeck tree was planted at the center, seasonal flowers were arranged along the curb edging, ornamental plants were added, and turf grass was installed as green ground cover</t>
+  </si>
+  <si>
+    <t>Following rehabilitation and site cleanup, Azadirachta indica trees were planted in an organized layout. Sand mounds were formed in selected areas, and various plants were introduced, including Thymus, Cymbopogon citratus, Bahraini basil, and mint. A curbside hedge of Bougainvillea was installed, with Sphagneticola trilobata used as ground cover</t>
+  </si>
+  <si>
+    <t>Planting beds were rehabilitated and upgraded in line with modern landscaping standards. Sustainable and ornamental species were introduced, including Tradescantia spathacea, Aloe vera, Agave, halfa grass, and Chlorophytum comosum, along with ground cover and ornamental trees to enhance the overall landscape</t>
+  </si>
+  <si>
+    <t>The soil and planting beds were rehabilitated, and ornamental trees were planted in an organized layout in line with modern landscaping standards</t>
+  </si>
+  <si>
+    <t>After soil preparation and installation of an irrigation system, ornamental trees and decorative plants were planted, seasonal flowers were added, and ground cover was installed to enhance the landscape</t>
+  </si>
+  <si>
+    <t>The land and soil were rehabilitated, ornamental trees were planted, and decorative plants and cacti were added within defined planting beds, along with appropriate ground cover to enhance the landscape</t>
+  </si>
+  <si>
+    <t>Previously: an old, woody, and deteriorated hedge of Volkameria inermis (wild jasmine).</t>
+  </si>
+  <si>
+    <t>Previously: mature Ficus microcarpa trees with degraded soil, invasive weeds, and agricultural debris.</t>
+  </si>
+  <si>
+    <t>Previously: overgrown and overlapping trees obstruct visibility and pose safety risks to pedestrians and drivers; some were dropping, woody, and visually appealing.</t>
+  </si>
+  <si>
+    <t>Previously: dry trees and invasive weeds negatively affecting the overall landscape appearance</t>
+  </si>
+  <si>
+    <t>Previously: randomly planted Conocarpus trees near the Ground Services Complex, with old woody and broken branches, invasive dry weeds, and agricultural debris across the site</t>
+  </si>
+  <si>
+    <t>Previously: scattered and dry trees, with old invasive weeds and debris within the planting areas</t>
+  </si>
+  <si>
+    <t>Previously: randomly planted Conocarpus trees with agricultural debris and invasive weeds on site</t>
+  </si>
+  <si>
+    <t>Western Gate Outer Roundabout</t>
   </si>
 </sst>
 </file>
@@ -953,7 +1019,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -990,14 +1056,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1335,23 +1393,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8" style="17" customWidth="1"/>
-    <col min="2" max="2" width="12" style="17" customWidth="1"/>
-    <col min="3" max="3" width="37" style="18" customWidth="1"/>
-    <col min="4" max="4" width="45" style="18" customWidth="1"/>
-    <col min="5" max="5" width="40" style="18" customWidth="1"/>
-    <col min="6" max="6" width="12" style="18" customWidth="1"/>
-    <col min="7" max="8" width="50" style="18" customWidth="1"/>
-    <col min="9" max="10" width="12" style="18" customWidth="1"/>
-    <col min="11" max="11" width="60" style="18" customWidth="1"/>
-    <col min="12" max="12" width="17.81640625" style="18" customWidth="1"/>
-    <col min="13" max="13" width="17.54296875" style="18" customWidth="1"/>
-    <col min="14" max="14" width="17.453125" style="18" customWidth="1"/>
-    <col min="15" max="15" width="17.7265625" style="18" customWidth="1"/>
-    <col min="16" max="16384" width="8.7265625" style="18"/>
+    <col min="1" max="1" width="8" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12" style="13" customWidth="1"/>
+    <col min="3" max="3" width="37" style="14" customWidth="1"/>
+    <col min="4" max="4" width="45" style="14" customWidth="1"/>
+    <col min="5" max="5" width="40" style="14" customWidth="1"/>
+    <col min="6" max="6" width="12" style="14" customWidth="1"/>
+    <col min="7" max="8" width="50" style="14" customWidth="1"/>
+    <col min="9" max="10" width="12" style="14" customWidth="1"/>
+    <col min="11" max="11" width="60" style="14" customWidth="1"/>
+    <col min="12" max="12" width="17.81640625" style="14" customWidth="1"/>
+    <col min="13" max="13" width="17.54296875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="17.453125" style="14" customWidth="1"/>
+    <col min="15" max="15" width="17.7265625" style="14" customWidth="1"/>
+    <col min="16" max="16384" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="2" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1411,7 +1469,7 @@
       <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="22" t="s">
         <v>12</v>
       </c>
       <c r="E2" s="4" t="s">
@@ -1446,7 +1504,7 @@
       <c r="C3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="22" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -1481,7 +1539,7 @@
       <c r="C4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="22" t="s">
         <v>26</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -1516,7 +1574,7 @@
       <c r="C5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="22" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -1551,7 +1609,7 @@
       <c r="C6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="22" t="s">
         <v>39</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -1586,7 +1644,7 @@
       <c r="C7" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="22" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -1621,7 +1679,7 @@
       <c r="C8" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="22" t="s">
         <v>54</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -1656,7 +1714,7 @@
       <c r="C9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="22" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1691,7 +1749,7 @@
       <c r="C10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="22" t="s">
         <v>67</v>
       </c>
       <c r="E10" s="4" t="s">
@@ -1726,7 +1784,7 @@
       <c r="C11" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="22" t="s">
         <v>73</v>
       </c>
       <c r="E11" s="4" t="s">
@@ -1761,7 +1819,7 @@
       <c r="C12" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="22" t="s">
         <v>80</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -1796,7 +1854,7 @@
       <c r="C13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="22" t="s">
         <v>87</v>
       </c>
       <c r="E13" s="4" t="s">
@@ -1831,7 +1889,7 @@
       <c r="C14" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="22" t="s">
         <v>95</v>
       </c>
       <c r="E14" s="4" t="s">
@@ -1866,7 +1924,7 @@
       <c r="C15" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="22" t="s">
         <v>102</v>
       </c>
       <c r="E15" s="4" t="s">
@@ -1901,7 +1959,7 @@
       <c r="C16" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="22" t="s">
         <v>107</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -1936,7 +1994,7 @@
       <c r="C17" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="22" t="s">
         <v>114</v>
       </c>
       <c r="E17" s="4" t="s">
@@ -1971,7 +2029,7 @@
       <c r="C18" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="22" t="s">
         <v>121</v>
       </c>
       <c r="E18" s="4" t="s">
@@ -2006,7 +2064,7 @@
       <c r="C19" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="22" t="s">
         <v>126</v>
       </c>
       <c r="E19" s="4" t="s">
@@ -2041,7 +2099,7 @@
       <c r="C20" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="22" t="s">
         <v>133</v>
       </c>
       <c r="E20" s="4" t="s">
@@ -2076,7 +2134,7 @@
       <c r="C21" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="22" t="s">
         <v>139</v>
       </c>
       <c r="E21" s="4" t="s">
@@ -2111,7 +2169,7 @@
       <c r="C22" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="D22" s="22" t="s">
         <v>145</v>
       </c>
       <c r="E22" s="4" t="s">
@@ -2146,7 +2204,7 @@
       <c r="C23" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="22" t="s">
         <v>149</v>
       </c>
       <c r="E23" s="4" t="s">
@@ -2181,7 +2239,7 @@
       <c r="C24" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="22" t="s">
         <v>153</v>
       </c>
       <c r="E24" s="4" t="s">
@@ -2216,7 +2274,7 @@
       <c r="C25" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="21" t="s">
         <v>159</v>
       </c>
       <c r="E25" s="7" t="s">
@@ -2251,7 +2309,7 @@
       <c r="C26" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="21" t="s">
         <v>166</v>
       </c>
       <c r="E26" s="7" t="s">
@@ -2286,7 +2344,7 @@
       <c r="C27" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="D27" s="21" t="s">
         <v>173</v>
       </c>
       <c r="E27" s="7" t="s">
@@ -2321,7 +2379,7 @@
       <c r="C28" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D28" s="25" t="s">
+      <c r="D28" s="21" t="s">
         <v>180</v>
       </c>
       <c r="E28" s="7" t="s">
@@ -2356,7 +2414,7 @@
       <c r="C29" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D29" s="25" t="s">
+      <c r="D29" s="21" t="s">
         <v>186</v>
       </c>
       <c r="E29" s="7" t="s">
@@ -2391,7 +2449,7 @@
       <c r="C30" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="D30" s="21" t="s">
         <v>193</v>
       </c>
       <c r="E30" s="7" t="s">
@@ -2426,7 +2484,7 @@
       <c r="C31" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="D31" s="25" t="s">
+      <c r="D31" s="21" t="s">
         <v>199</v>
       </c>
       <c r="E31" s="7" t="s">
@@ -2461,7 +2519,7 @@
       <c r="C32" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" s="21" t="s">
         <v>206</v>
       </c>
       <c r="E32" s="7" t="s">
@@ -2496,7 +2554,7 @@
       <c r="C33" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="21" t="s">
         <v>212</v>
       </c>
       <c r="E33" s="7" t="s">
@@ -2531,7 +2589,7 @@
       <c r="C34" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="D34" s="25" t="s">
+      <c r="D34" s="21" t="s">
         <v>217</v>
       </c>
       <c r="E34" s="7" t="s">
@@ -2566,7 +2624,7 @@
       <c r="C35" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="D35" s="25" t="s">
+      <c r="D35" s="21" t="s">
         <v>224</v>
       </c>
       <c r="E35" s="7" t="s">
@@ -2591,7 +2649,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="36" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" s="12" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A36" s="9">
         <v>2026</v>
       </c>
@@ -2604,9 +2662,17 @@
       <c r="D36" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="E36" s="10"/>
-    </row>
-    <row r="37" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="E36" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" s="12" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A37" s="9">
         <v>2026</v>
       </c>
@@ -2619,9 +2685,17 @@
       <c r="D37" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="E37" s="10"/>
-    </row>
-    <row r="38" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="E37" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" s="12" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A38" s="9">
         <v>2026</v>
       </c>
@@ -2635,8 +2709,14 @@
         <v>240</v>
       </c>
       <c r="E38" s="10"/>
-    </row>
-    <row r="39" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G38" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" s="12" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A39" s="9">
         <v>2026</v>
       </c>
@@ -2650,23 +2730,35 @@
         <v>244</v>
       </c>
       <c r="E39" s="10"/>
-    </row>
-    <row r="40" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="13">
+      <c r="G39" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" s="12" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A40" s="9">
         <v>2026</v>
       </c>
       <c r="B40" s="9">
         <v>5</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="C40" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="E40" s="14"/>
-    </row>
-    <row r="41" spans="1:11" s="12" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="E40" s="10"/>
+      <c r="G40" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="H40" s="12" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" s="12" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A41" s="9">
         <v>2026</v>
       </c>
@@ -2680,8 +2772,14 @@
         <v>247</v>
       </c>
       <c r="E41" s="10"/>
-    </row>
-    <row r="42" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G41" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" s="12" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A42" s="9">
         <v>2026</v>
       </c>
@@ -2695,8 +2793,14 @@
         <v>248</v>
       </c>
       <c r="E42" s="10"/>
-    </row>
-    <row r="43" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G42" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" s="12" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="9">
         <v>2026</v>
       </c>
@@ -2706,12 +2810,18 @@
       <c r="C43" s="12" t="s">
         <v>255</v>
       </c>
-      <c r="D43" s="23" t="s">
+      <c r="D43" s="19" t="s">
         <v>264</v>
       </c>
       <c r="E43" s="10"/>
-    </row>
-    <row r="44" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G43" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" s="12" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A44" s="9">
         <v>2026</v>
       </c>
@@ -2721,12 +2831,18 @@
       <c r="C44" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="D44" s="23" t="s">
+      <c r="D44" s="19" t="s">
         <v>266</v>
       </c>
       <c r="E44" s="10"/>
-    </row>
-    <row r="45" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G44" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" s="12" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A45" s="9">
         <v>2026</v>
       </c>
@@ -2736,176 +2852,195 @@
       <c r="C45" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="D45" s="23" t="s">
+      <c r="D45" s="19" t="s">
         <v>224</v>
       </c>
       <c r="E45" s="10"/>
-    </row>
-    <row r="46" spans="1:11" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="19">
+      <c r="G45" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="H45" s="12" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="9">
+        <v>2026</v>
+      </c>
+      <c r="B46" s="9">
+        <v>11</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="D46" s="19"/>
+      <c r="E46" s="10"/>
+    </row>
+    <row r="47" spans="1:11" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="15">
         <v>2027</v>
       </c>
-      <c r="B46" s="19">
+      <c r="B47" s="15">
         <v>1</v>
       </c>
-      <c r="C46" s="20" t="s">
+      <c r="C47" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D47" s="17" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="47" spans="1:11" s="22" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A47" s="19">
+    <row r="48" spans="1:11" s="18" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A48" s="15">
         <v>2027</v>
       </c>
-      <c r="B47" s="19">
+      <c r="B48" s="15">
         <v>2</v>
       </c>
-      <c r="C47" s="20" t="s">
+      <c r="C48" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D48" s="17" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="48" spans="1:11" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="19">
+    <row r="49" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="15">
         <v>2027</v>
       </c>
-      <c r="B48" s="19">
+      <c r="B49" s="15">
         <v>3</v>
       </c>
-      <c r="C48" s="20" t="s">
+      <c r="C49" s="16" t="s">
         <v>233</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="D49" s="17" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="49" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="19">
+    <row r="50" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="15">
         <v>2027</v>
       </c>
-      <c r="B49" s="19">
+      <c r="B50" s="15">
         <v>4</v>
       </c>
-      <c r="C49" s="20" t="s">
+      <c r="C50" s="16" t="s">
         <v>263</v>
       </c>
-      <c r="D49" s="21" t="s">
+      <c r="D50" s="17" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="50" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="19">
+    <row r="51" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="15">
         <v>2027</v>
       </c>
-      <c r="B50" s="19">
+      <c r="B51" s="15">
         <v>5</v>
       </c>
-      <c r="C50" s="20" t="s">
+      <c r="C51" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="D51" s="17" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="51" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="19">
+    <row r="52" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="15">
         <v>2027</v>
       </c>
-      <c r="B51" s="19">
+      <c r="B52" s="15">
         <v>6</v>
       </c>
-      <c r="C51" s="20" t="s">
+      <c r="C52" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="D51" s="21" t="s">
+      <c r="D52" s="17" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="52" spans="1:4" s="22" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A52" s="19">
+    <row r="53" spans="1:4" s="18" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="15">
         <v>2027</v>
       </c>
-      <c r="B52" s="19">
+      <c r="B53" s="15">
         <v>7</v>
       </c>
-      <c r="C52" s="20" t="s">
+      <c r="C53" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D53" s="17" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="53" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="19">
+    <row r="54" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="15">
         <v>2027</v>
       </c>
-      <c r="B53" s="19">
+      <c r="B54" s="15">
         <v>8</v>
       </c>
-      <c r="C53" s="20" t="s">
+      <c r="C54" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="D53" s="21" t="s">
+      <c r="D54" s="17" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="54" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="19">
+    <row r="55" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="15">
         <v>2027</v>
       </c>
-      <c r="B54" s="19">
+      <c r="B55" s="15">
         <v>9</v>
       </c>
-      <c r="C54" s="22" t="s">
+      <c r="C55" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="D54" s="24" t="s">
+      <c r="D55" s="20" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="55" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="19">
+    <row r="56" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="15">
         <v>2027</v>
       </c>
-      <c r="B55" s="19">
+      <c r="B56" s="15">
         <v>10</v>
       </c>
-      <c r="C55" s="22" t="s">
+      <c r="C56" s="18" t="s">
         <v>258</v>
       </c>
-      <c r="D55" s="24" t="s">
+      <c r="D56" s="20" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="56" spans="1:4" s="22" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A56" s="19">
+    <row r="57" spans="1:4" s="18" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="15">
         <v>2027</v>
       </c>
-      <c r="B56" s="19">
+      <c r="B57" s="15">
         <v>11</v>
       </c>
-      <c r="C56" s="22" t="s">
+      <c r="C57" s="18" t="s">
         <v>259</v>
       </c>
-      <c r="D56" s="24" t="s">
+      <c r="D57" s="20" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="57" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="19">
+    <row r="58" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="15">
         <v>2027</v>
       </c>
-      <c r="B57" s="19">
+      <c r="B58" s="15">
         <v>12</v>
       </c>
-      <c r="C57" s="22" t="s">
+      <c r="C58" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="D57" s="24" t="s">
+      <c r="D58" s="20" t="s">
         <v>269</v>
       </c>
     </row>
@@ -2914,24 +3049,24 @@
     <hyperlink ref="D36" r:id="rId1" xr:uid="{1000462C-B238-431A-B2A1-3FC2BD2E2813}"/>
     <hyperlink ref="D37" r:id="rId2" xr:uid="{1B9305A2-EFAE-494D-AE61-72B82236A00A}"/>
     <hyperlink ref="D38" r:id="rId3" xr:uid="{37366389-41FF-4E4B-BBAA-23F6E2BDE2E5}"/>
-    <hyperlink ref="D47" r:id="rId4" xr:uid="{0D35B99D-C761-48D2-A6FC-1AA9DABC570E}"/>
-    <hyperlink ref="D48" r:id="rId5" xr:uid="{2C3EF60F-AF56-486A-A65A-90521D1BE076}"/>
+    <hyperlink ref="D48" r:id="rId4" xr:uid="{0D35B99D-C761-48D2-A6FC-1AA9DABC570E}"/>
+    <hyperlink ref="D49" r:id="rId5" xr:uid="{2C3EF60F-AF56-486A-A65A-90521D1BE076}"/>
     <hyperlink ref="D39" r:id="rId6" xr:uid="{C95DBB32-C8B9-4192-B5A8-A2BBC5AE8709}"/>
-    <hyperlink ref="D49" r:id="rId7" xr:uid="{0245B09C-A05C-42F8-9F53-B3C0DF8A3B3B}"/>
+    <hyperlink ref="D50" r:id="rId7" xr:uid="{0245B09C-A05C-42F8-9F53-B3C0DF8A3B3B}"/>
     <hyperlink ref="D40" r:id="rId8" xr:uid="{41838A62-16DE-40C3-A6D6-65FCB68C828C}"/>
     <hyperlink ref="D41" r:id="rId9" xr:uid="{1DA3C22A-9C35-431D-9E54-09A3B7395A7F}"/>
     <hyperlink ref="D42" r:id="rId10" xr:uid="{D058C4E8-F8D4-42F8-A17C-BC9F6C69C57E}"/>
-    <hyperlink ref="D50" r:id="rId11" xr:uid="{D2DB956F-0AE2-4C2E-8230-86EBD2EFD849}"/>
-    <hyperlink ref="D51" r:id="rId12" xr:uid="{7FDA2993-EE4C-4AEE-A744-BD17EE8DF685}"/>
-    <hyperlink ref="D52" r:id="rId13" xr:uid="{C3597594-CEFA-42FD-809C-D15002498BB3}"/>
-    <hyperlink ref="D53" r:id="rId14" xr:uid="{D97DA6E9-7A4E-4C31-A094-581BEFAE38C5}"/>
-    <hyperlink ref="D46" r:id="rId15" xr:uid="{66A90A50-7813-4BE2-835B-908012476FD3}"/>
+    <hyperlink ref="D51" r:id="rId11" xr:uid="{D2DB956F-0AE2-4C2E-8230-86EBD2EFD849}"/>
+    <hyperlink ref="D52" r:id="rId12" xr:uid="{7FDA2993-EE4C-4AEE-A744-BD17EE8DF685}"/>
+    <hyperlink ref="D53" r:id="rId13" xr:uid="{C3597594-CEFA-42FD-809C-D15002498BB3}"/>
+    <hyperlink ref="D54" r:id="rId14" xr:uid="{D97DA6E9-7A4E-4C31-A094-581BEFAE38C5}"/>
+    <hyperlink ref="D47" r:id="rId15" xr:uid="{66A90A50-7813-4BE2-835B-908012476FD3}"/>
     <hyperlink ref="D43" r:id="rId16" xr:uid="{147ACBB0-7330-4375-A5F5-59953D8672C7}"/>
-    <hyperlink ref="D54" r:id="rId17" xr:uid="{BFA2C4D2-299F-48F3-8C92-FA17876C33A6}"/>
+    <hyperlink ref="D55" r:id="rId17" xr:uid="{BFA2C4D2-299F-48F3-8C92-FA17876C33A6}"/>
     <hyperlink ref="D44" r:id="rId18" xr:uid="{89B226A2-CD02-441A-9332-0B81D06E4B1B}"/>
-    <hyperlink ref="D55" r:id="rId19" xr:uid="{0455FD2A-FBB6-4033-952F-93501D724B92}"/>
-    <hyperlink ref="D56" r:id="rId20" xr:uid="{6900060F-FF2A-4358-B515-6B63FC613431}"/>
-    <hyperlink ref="D57" r:id="rId21" xr:uid="{57F6A3F4-C756-45F7-BF88-FF8069986A7A}"/>
+    <hyperlink ref="D56" r:id="rId19" xr:uid="{0455FD2A-FBB6-4033-952F-93501D724B92}"/>
+    <hyperlink ref="D57" r:id="rId20" xr:uid="{6900060F-FF2A-4358-B515-6B63FC613431}"/>
+    <hyperlink ref="D58" r:id="rId21" xr:uid="{57F6A3F4-C756-45F7-BF88-FF8069986A7A}"/>
     <hyperlink ref="D35" r:id="rId22" xr:uid="{D5D38438-E4B6-481E-8C69-DFDC27DE2CD2}"/>
     <hyperlink ref="D45" r:id="rId23" xr:uid="{A775D76D-67D0-401B-BFFA-3EBAA24D153A}"/>
     <hyperlink ref="D34" r:id="rId24" xr:uid="{A2DE1ABB-0FFA-4088-A49E-6A441A99A49F}"/>

</xml_diff>